<commit_message>
Update ils-postplanner-2026-04-13.xlsx (regenerated during April 14 pipeline run)
https://claude.ai/code/session_01WqM2kYprBN1KHUykJafuQB
</commit_message>
<xml_diff>
--- a/Softball/postplanner-imports/ils-postplanner-2026-04-13.xlsx
+++ b/Softball/postplanner-imports/ils-postplanner-2026-04-13.xlsx
@@ -478,7 +478,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>04/13/2026  11:07</t>
+          <t>04/13/2026  09:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -493,7 +493,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>04/13/2026  11:36</t>
+          <t>04/13/2026  09:05</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -507,7 +507,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>04/13/2026  12:05</t>
+          <t>04/13/2026  09:10</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -523,7 +523,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04/13/2026  12:34</t>
+          <t>04/13/2026  09:15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -535,7 +535,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04/13/2026  13:03</t>
+          <t>04/13/2026  09:20</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -553,7 +553,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04/13/2026  13:32</t>
+          <t>04/13/2026  09:25</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -565,7 +565,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04/13/2026  14:01</t>
+          <t>04/13/2026  11:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -579,7 +579,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04/13/2026  14:30</t>
+          <t>04/13/2026  11:05</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -596,7 +596,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04/13/2026  14:59</t>
+          <t>04/13/2026  11:10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -608,7 +608,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04/13/2026  15:28</t>
+          <t>04/13/2026  13:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -623,7 +623,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04/13/2026  15:57</t>
+          <t>04/13/2026  15:00</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -638,7 +638,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04/13/2026  16:26</t>
+          <t>04/13/2026  15:05</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -654,7 +654,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>04/13/2026  16:55</t>
+          <t>04/13/2026  15:10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -666,7 +666,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04/13/2026  17:24</t>
+          <t>04/13/2026  17:30</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -680,7 +680,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04/13/2026  17:53</t>
+          <t>04/13/2026  17:35</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -696,7 +696,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>04/13/2026  18:22</t>
+          <t>04/13/2026  17:40</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -708,7 +708,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>04/13/2026  18:51</t>
+          <t>04/13/2026  20:00</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -722,7 +722,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>04/13/2026  19:20</t>
+          <t>04/13/2026  20:05</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -738,7 +738,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>04/13/2026  19:49</t>
+          <t>04/13/2026  20:10</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -753,7 +753,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>04/13/2026  20:18</t>
+          <t>04/13/2026  20:15</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -765,7 +765,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>04/13/2026  20:47</t>
+          <t>04/13/2026  20:20</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -782,7 +782,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>04/13/2026  21:16</t>
+          <t>04/13/2026  20:25</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">

</xml_diff>